<commit_message>
Add complaint templates, evidence checklist, and 35 test scenarios
</commit_message>
<xml_diff>
--- a/legal_aid_centers.xlsx
+++ b/legal_aid_centers.xlsx
@@ -862,35 +862,35 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1155,8 +1155,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>